<commit_message>
BOM changes done (supplier and eSpark) #151
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Bottom Board/_BOM/Supplier BOM_Bottom (20 Boards).xlsx
+++ b/Deliverables/SM_Bottom Board/_BOM/Supplier BOM_Bottom (20 Boards).xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Faizan\GitHub\ColeBenson-SmartMotors\Deliverables\SM_Bottom Board\_BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Faizan\GitHub\ColeBenson-SmartMotors\Deliverables\SM_Bottom Board\_BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="188">
   <si>
     <t>Component list</t>
   </si>
@@ -208,9 +208,6 @@
     <t>IC TRANSCEIVER 1/1 8SOIC</t>
   </si>
   <si>
-    <t>WIDE-FULL SCALE RANGE 6-AXIS MEM</t>
-  </si>
-  <si>
     <t>IC BUF NON-INVERT 5.5V SOT23-5</t>
   </si>
   <si>
@@ -271,9 +268,6 @@
     <t>SOIC-8</t>
   </si>
   <si>
-    <t>24-QFN (3x3)</t>
-  </si>
-  <si>
     <t>SOT-23-5</t>
   </si>
   <si>
@@ -325,9 +319,6 @@
     <t>RC0603FR-07470RL</t>
   </si>
   <si>
-    <t>ICM-20649</t>
-  </si>
-  <si>
     <t>SN74LV1T34DBVR</t>
   </si>
   <si>
@@ -374,9 +365,6 @@
   </si>
   <si>
     <t>Texas Instruments</t>
-  </si>
-  <si>
-    <t>TDK InvenSense</t>
   </si>
   <si>
     <t>Microchip</t>
@@ -609,11 +597,20 @@
   <si>
     <t>PG-DSO-8 Position Sensor ROHS</t>
   </si>
+  <si>
+    <t>LGA-14 Attitude Sensor/Gyroscope</t>
+  </si>
+  <si>
+    <t>LGA-14</t>
+  </si>
+  <si>
+    <t>LSM6DSLTR</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
@@ -629,6 +626,7 @@
       <sz val="10"/>
       <color indexed="13"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -1285,7 +1283,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1584,23 +1582,23 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:L44"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="3.1796875" style="25" customWidth="1"/>
-    <col min="3" max="3" width="18.7265625" style="25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" style="25" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="26.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.7265625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.81640625" customWidth="1"/>
-    <col min="12" max="12" width="29.453125" customWidth="1"/>
-    <col min="14" max="14" width="18.26953125" customWidth="1"/>
+    <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.85546875" customWidth="1"/>
+    <col min="12" max="12" width="29.42578125" customWidth="1"/>
+    <col min="14" max="14" width="18.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -1614,7 +1612,7 @@
       <c r="K1" s="72"/>
       <c r="L1" s="72"/>
     </row>
-    <row r="2" spans="1:12" ht="31.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:12" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="20"/>
       <c r="C2" s="46"/>
@@ -1632,7 +1630,7 @@
       <c r="K2" s="3"/>
       <c r="L2" s="43"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="21"/>
       <c r="C3" s="47"/>
@@ -1650,7 +1648,7 @@
       <c r="K3" s="4"/>
       <c r="L3" s="73"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="21"/>
       <c r="C4" s="47"/>
@@ -1668,7 +1666,7 @@
       <c r="K4" s="6"/>
       <c r="L4" s="74"/>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="21"/>
       <c r="C5" s="47"/>
@@ -1686,7 +1684,7 @@
       <c r="K5" s="5"/>
       <c r="L5" s="74"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="22"/>
       <c r="C6" s="48"/>
@@ -1700,7 +1698,7 @@
       <c r="K6" s="5"/>
       <c r="L6" s="74"/>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="23"/>
       <c r="C7" s="49"/>
@@ -1714,7 +1712,7 @@
       <c r="K7" s="7"/>
       <c r="L7" s="74"/>
     </row>
-    <row r="8" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="26"/>
       <c r="C8" s="50"/>
@@ -1728,13 +1726,13 @@
       <c r="K8" s="7"/>
       <c r="L8" s="74"/>
     </row>
-    <row r="9" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="29" t="s">
         <v>4</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="D9" s="29" t="s">
         <v>10</v>
@@ -1743,35 +1741,35 @@
         <v>40</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="H9" s="29" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="J9" s="29" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="K9" s="29" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="L9" s="31" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="53">
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
       <c r="C10" s="37" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="D10" s="37" t="s">
         <v>11</v>
@@ -1780,16 +1778,16 @@
         <v>41</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G10" s="38" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="H10" s="37" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="I10" s="38" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="J10" s="37">
         <v>1</v>
@@ -1800,32 +1798,32 @@
       </c>
       <c r="L10" s="41"/>
     </row>
-    <row r="11" spans="1:12" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="53">
         <f t="shared" ref="B11:B41" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="39" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="D11" s="39" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="E11" s="40" t="s">
         <v>42</v>
       </c>
       <c r="F11" s="39" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G11" s="40" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="H11" s="39" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="I11" s="40" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="J11" s="65">
         <v>18</v>
@@ -1835,35 +1833,35 @@
         <v>360</v>
       </c>
       <c r="L11" s="68" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="53">
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
       <c r="C12" s="37" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="D12" s="37" t="s">
         <v>12</v>
       </c>
       <c r="E12" s="38" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="F12" s="37" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="G12" s="38" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="H12" s="37" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="I12" s="38" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="J12" s="37">
         <v>1</v>
@@ -1874,14 +1872,14 @@
       </c>
       <c r="L12" s="61"/>
     </row>
-    <row r="13" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="53">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C13" s="39" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="D13" s="39" t="s">
         <v>13</v>
@@ -1890,16 +1888,16 @@
         <v>43</v>
       </c>
       <c r="F13" s="39" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G13" s="40" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H13" s="39" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="I13" s="40" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="J13" s="39">
         <v>2</v>
@@ -1910,14 +1908,14 @@
       </c>
       <c r="L13" s="42"/>
     </row>
-    <row r="14" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="53">
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
       </c>
       <c r="C14" s="37" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="D14" s="37" t="s">
         <v>14</v>
@@ -1926,16 +1924,16 @@
         <v>44</v>
       </c>
       <c r="F14" s="37" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G14" s="38" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="H14" s="37" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="I14" s="38" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="J14" s="37">
         <v>2</v>
@@ -1946,32 +1944,32 @@
       </c>
       <c r="L14" s="41"/>
     </row>
-    <row r="15" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="53">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C15" s="39" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="D15" s="39" t="s">
         <v>15</v>
       </c>
       <c r="E15" s="40" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="F15" s="39" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G15" s="39" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="H15" s="39" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="I15" s="40" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="J15" s="39">
         <v>2</v>
@@ -1982,14 +1980,14 @@
       </c>
       <c r="L15" s="42"/>
     </row>
-    <row r="16" spans="1:12" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="53">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="C16" s="39" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="D16" s="39" t="s">
         <v>16</v>
@@ -1998,16 +1996,16 @@
         <v>42</v>
       </c>
       <c r="F16" s="39" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G16" s="40" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="H16" s="39" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="I16" s="40" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="J16" s="39">
         <v>1</v>
@@ -2018,32 +2016,32 @@
       </c>
       <c r="L16" s="42"/>
     </row>
-    <row r="17" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="53">
         <f>ROW(B17) - ROW($B$9)</f>
         <v>8</v>
       </c>
       <c r="C17" s="37" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D17" s="37" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="E17" s="38" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="F17" s="37" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G17" s="37" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="H17" s="37" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="I17" s="38" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="J17" s="62">
         <v>1</v>
@@ -2054,14 +2052,14 @@
       </c>
       <c r="L17" s="61"/>
     </row>
-    <row r="18" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="53">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="C18" s="39" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D18" s="39" t="s">
         <v>17</v>
@@ -2070,16 +2068,16 @@
         <v>45</v>
       </c>
       <c r="F18" s="39" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G18" s="40" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="H18" s="39" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="I18" s="40" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="J18" s="39">
         <v>1</v>
@@ -2090,14 +2088,14 @@
       </c>
       <c r="L18" s="42"/>
     </row>
-    <row r="19" spans="1:12" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="53">
         <f>ROW(B19) - ROW($B$9)</f>
         <v>10</v>
       </c>
       <c r="C19" s="37" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D19" s="37" t="s">
         <v>18</v>
@@ -2106,16 +2104,16 @@
         <v>46</v>
       </c>
       <c r="F19" s="37" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="G19" s="38" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H19" s="37" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="I19" s="38" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="J19" s="37">
         <v>4</v>
@@ -2126,14 +2124,14 @@
       </c>
       <c r="L19" s="41"/>
     </row>
-    <row r="20" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="53">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="C20" s="39" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="D20" s="39" t="s">
         <v>19</v>
@@ -2142,16 +2140,16 @@
         <v>47</v>
       </c>
       <c r="F20" s="39" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="G20" s="40" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H20" s="39" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="I20" s="40" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="J20" s="39">
         <v>1</v>
@@ -2162,14 +2160,14 @@
       </c>
       <c r="L20" s="42"/>
     </row>
-    <row r="21" spans="1:12" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="53">
         <f>ROW(B21) - ROW($B$9)</f>
         <v>12</v>
       </c>
       <c r="C21" s="37" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D21" s="37" t="s">
         <v>20</v>
@@ -2178,16 +2176,16 @@
         <v>48</v>
       </c>
       <c r="F21" s="37" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G21" s="38" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H21" s="37" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="I21" s="38" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="J21" s="37">
         <v>1</v>
@@ -2198,14 +2196,14 @@
       </c>
       <c r="L21" s="41"/>
     </row>
-    <row r="22" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="53">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="C22" s="39" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="D22" s="39" t="s">
         <v>21</v>
@@ -2214,16 +2212,16 @@
         <v>49</v>
       </c>
       <c r="F22" s="39" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G22" s="39" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="H22" s="39" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="I22" s="40" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="J22" s="39">
         <v>1</v>
@@ -2234,14 +2232,14 @@
       </c>
       <c r="L22" s="42"/>
     </row>
-    <row r="23" spans="1:12" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:12" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="53">
         <f>ROW(B23) - ROW($B$9)</f>
         <v>14</v>
       </c>
       <c r="C23" s="37" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="D23" s="37" t="s">
         <v>22</v>
@@ -2250,16 +2248,16 @@
         <v>50</v>
       </c>
       <c r="F23" s="37" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="G23" s="38" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H23" s="37" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="I23" s="38" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="J23" s="37">
         <v>1</v>
@@ -2270,14 +2268,14 @@
       </c>
       <c r="L23" s="41"/>
     </row>
-    <row r="24" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="53">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="C24" s="39" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="D24" s="39" t="s">
         <v>23</v>
@@ -2286,16 +2284,16 @@
         <v>51</v>
       </c>
       <c r="F24" s="39" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G24" s="40" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="H24" s="39" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="I24" s="40" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="J24" s="39">
         <v>2</v>
@@ -2306,14 +2304,14 @@
       </c>
       <c r="L24" s="42"/>
     </row>
-    <row r="25" spans="1:12" ht="48.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:12" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="53">
         <f>ROW(B25) - ROW($B$9)</f>
         <v>16</v>
       </c>
       <c r="C25" s="37" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D25" s="37" t="s">
         <v>24</v>
@@ -2322,16 +2320,16 @@
         <v>52</v>
       </c>
       <c r="F25" s="37" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G25" s="38" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="H25" s="37" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="I25" s="38" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="J25" s="37">
         <v>40</v>
@@ -2342,14 +2340,14 @@
       </c>
       <c r="L25" s="41"/>
     </row>
-    <row r="26" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="53">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="C26" s="39" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D26" s="39" t="s">
         <v>25</v>
@@ -2358,16 +2356,16 @@
         <v>53</v>
       </c>
       <c r="F26" s="39" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G26" s="40" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H26" s="39" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="I26" s="40" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="J26" s="39">
         <v>7</v>
@@ -2378,32 +2376,32 @@
       </c>
       <c r="L26" s="42"/>
     </row>
-    <row r="27" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="53">
         <f>ROW(B27) - ROW($B$9)</f>
         <v>18</v>
       </c>
       <c r="C27" s="37" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D27" s="37" t="s">
         <v>26</v>
       </c>
       <c r="E27" s="38" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="F27" s="37" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G27" s="38" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="H27" s="37" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="I27" s="38" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="J27" s="37">
         <v>1</v>
@@ -2414,14 +2412,14 @@
       </c>
       <c r="L27" s="41"/>
     </row>
-    <row r="28" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="53">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="C28" s="39" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D28" s="39" t="s">
         <v>27</v>
@@ -2430,16 +2428,16 @@
         <v>54</v>
       </c>
       <c r="F28" s="39" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G28" s="40" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="H28" s="39" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="I28" s="40" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="J28" s="39">
         <v>2</v>
@@ -2450,32 +2448,32 @@
       </c>
       <c r="L28" s="42"/>
     </row>
-    <row r="29" spans="1:12" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="53">
         <f>ROW(B29) - ROW($B$9)</f>
         <v>20</v>
       </c>
       <c r="C29" s="37" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D29" s="66" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="E29" s="38" t="s">
         <v>55</v>
       </c>
       <c r="F29" s="37" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G29" s="38" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="H29" s="37" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="I29" s="38" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="J29" s="67">
         <v>2</v>
@@ -2485,35 +2483,35 @@
         <v>40</v>
       </c>
       <c r="L29" s="61" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="53">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="C30" s="39" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D30" s="39" t="s">
         <v>28</v>
       </c>
       <c r="E30" s="40" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="F30" s="39" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G30" s="39" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="H30" s="39" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="I30" s="40" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="J30" s="39">
         <v>2</v>
@@ -2524,31 +2522,31 @@
       </c>
       <c r="L30" s="42"/>
     </row>
-    <row r="31" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="53">
         <v>22</v>
       </c>
       <c r="C31" s="69" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D31" s="64" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="E31" s="70" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="F31" s="64" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G31" s="70" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="H31" s="64" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="I31" s="70" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="J31" s="64">
         <v>2</v>
@@ -2558,17 +2556,17 @@
         <v>40</v>
       </c>
       <c r="L31" s="71" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="32" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="53">
         <f>ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
       <c r="C32" s="58" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D32" s="58" t="s">
         <v>29</v>
@@ -2577,16 +2575,16 @@
         <v>56</v>
       </c>
       <c r="F32" s="58" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G32" s="59" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="H32" s="58" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="I32" s="59" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="J32" s="58">
         <v>8</v>
@@ -2596,35 +2594,35 @@
         <v>160</v>
       </c>
       <c r="L32" s="60" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="33" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="53">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="C33" s="39" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="D33" s="39" t="s">
         <v>30</v>
       </c>
       <c r="E33" s="40" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="F33" s="39" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="G33" s="39" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="H33" s="39" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="I33" s="40" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="J33" s="39">
         <v>1</v>
@@ -2635,14 +2633,14 @@
       </c>
       <c r="L33" s="63"/>
     </row>
-    <row r="34" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="53">
         <f>ROW(B34) - ROW($B$9)</f>
         <v>25</v>
       </c>
       <c r="C34" s="37" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D34" s="37" t="s">
         <v>31</v>
@@ -2651,16 +2649,16 @@
         <v>57</v>
       </c>
       <c r="F34" s="37" t="s">
+        <v>142</v>
+      </c>
+      <c r="G34" s="38" t="s">
+        <v>181</v>
+      </c>
+      <c r="H34" s="37" t="s">
+        <v>110</v>
+      </c>
+      <c r="I34" s="38" t="s">
         <v>146</v>
-      </c>
-      <c r="G34" s="38" t="s">
-        <v>185</v>
-      </c>
-      <c r="H34" s="37" t="s">
-        <v>113</v>
-      </c>
-      <c r="I34" s="38" t="s">
-        <v>150</v>
       </c>
       <c r="J34" s="37">
         <v>1</v>
@@ -2670,17 +2668,17 @@
         <v>20</v>
       </c>
       <c r="L34" s="61" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="53">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
       <c r="C35" s="39" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D35" s="39" t="s">
         <v>32</v>
@@ -2689,16 +2687,16 @@
         <v>58</v>
       </c>
       <c r="F35" s="39" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G35" s="39" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="H35" s="39" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="I35" s="40" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="J35" s="39">
         <v>1</v>
@@ -2709,32 +2707,32 @@
       </c>
       <c r="L35" s="63"/>
     </row>
-    <row r="36" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="53">
         <f>ROW(B36) - ROW($B$9)</f>
         <v>27</v>
       </c>
       <c r="C36" s="37" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D36" s="37" t="s">
         <v>33</v>
       </c>
       <c r="E36" s="38" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="F36" s="37" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="G36" s="37" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="H36" s="37" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="I36" s="38" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="J36" s="37">
         <v>1</v>
@@ -2745,32 +2743,32 @@
       </c>
       <c r="L36" s="61"/>
     </row>
-    <row r="37" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="53">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
       <c r="C37" s="39" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D37" s="39" t="s">
         <v>34</v>
       </c>
       <c r="E37" s="40" t="s">
-        <v>59</v>
+        <v>185</v>
       </c>
       <c r="F37" s="39" t="s">
-        <v>80</v>
-      </c>
-      <c r="G37" s="40" t="s">
-        <v>98</v>
+        <v>186</v>
+      </c>
+      <c r="G37" s="39" t="s">
+        <v>187</v>
       </c>
       <c r="H37" s="39" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="I37" s="40" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="J37" s="39">
         <v>1</v>
@@ -2781,32 +2779,32 @@
       </c>
       <c r="L37" s="42"/>
     </row>
-    <row r="38" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="53">
         <f>ROW(B38) - ROW($B$9)</f>
         <v>29</v>
       </c>
       <c r="C38" s="37" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D38" s="37" t="s">
         <v>35</v>
       </c>
       <c r="E38" s="38" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F38" s="37" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G38" s="38" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="H38" s="37" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="I38" s="38" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="J38" s="37">
         <v>1</v>
@@ -2817,32 +2815,32 @@
       </c>
       <c r="L38" s="41"/>
     </row>
-    <row r="39" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="B39" s="53">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="C39" s="39" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D39" s="39" t="s">
         <v>36</v>
       </c>
       <c r="E39" s="40" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F39" s="39" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G39" s="40" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="H39" s="39" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="I39" s="40" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="J39" s="39">
         <v>1</v>
@@ -2853,32 +2851,32 @@
       </c>
       <c r="L39" s="42"/>
     </row>
-    <row r="40" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
       <c r="B40" s="53">
         <f>ROW(B40) - ROW($B$9)</f>
         <v>31</v>
       </c>
       <c r="C40" s="37" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D40" s="37" t="s">
         <v>37</v>
       </c>
       <c r="E40" s="38" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F40" s="37" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G40" s="38" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="H40" s="37" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="I40" s="38" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="J40" s="37">
         <v>1</v>
@@ -2889,32 +2887,32 @@
       </c>
       <c r="L40" s="41"/>
     </row>
-    <row r="41" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
       <c r="B41" s="53">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="C41" s="39" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="D41" s="39" t="s">
         <v>38</v>
       </c>
       <c r="E41" s="40" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F41" s="39" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="G41" s="40" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="H41" s="39" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="I41" s="40" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="J41" s="39">
         <v>1</v>
@@ -2925,32 +2923,32 @@
       </c>
       <c r="L41" s="42"/>
     </row>
-    <row r="42" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
       <c r="B42" s="53">
         <f>ROW(B42) - ROW($B$9)</f>
         <v>33</v>
       </c>
       <c r="C42" s="37" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="D42" s="37" t="s">
         <v>39</v>
       </c>
       <c r="E42" s="38" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F42" s="37" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="G42" s="38" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="H42" s="37" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="I42" s="38" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="J42" s="37">
         <v>1</v>
@@ -2961,7 +2959,7 @@
       </c>
       <c r="L42" s="41"/>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
       <c r="B43" s="32"/>
       <c r="C43" s="51"/>
@@ -2977,7 +2975,7 @@
       <c r="K43" s="36"/>
       <c r="L43" s="44"/>
     </row>
-    <row r="44" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
       <c r="B44" s="24"/>
       <c r="C44" s="52"/>

</xml_diff>

<commit_message>
corrections in supplier BOM
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Bottom Board/_BOM/Supplier BOM_Bottom (20 Boards).xlsx
+++ b/Deliverables/SM_Bottom Board/_BOM/Supplier BOM_Bottom (20 Boards).xlsx
@@ -1,26 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25831"/>
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Faizan\GitHub\ColeBenson-SmartMotors\Deliverables\SM_Bottom Board\_BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74D5B6B3-999F-4D4F-B05A-0ABF0B447455}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="179">
   <si>
     <t>Component list</t>
   </si>
@@ -469,9 +468,6 @@
     <t>RES SMD 100 OHM 1% 1/10W 0603</t>
   </si>
   <si>
-    <t>Multiple options added for MCU</t>
-  </si>
-  <si>
     <t>Nexperia</t>
   </si>
   <si>
@@ -496,24 +492,15 @@
     <t>CAP CER 10PF 25V C0G 0201</t>
   </si>
   <si>
-    <t>CGA1A2C0G1E100D030BA</t>
-  </si>
-  <si>
     <t>TVS DIODE 24VWM 41VC TO236AB</t>
   </si>
   <si>
-    <t>XZVG68W-2</t>
-  </si>
-  <si>
     <t>SunLED</t>
   </si>
   <si>
     <t>Res Thick Film 0201 806 Ohm 1% 1/20W ±200ppm/°C Molded SMD SMD Paper T/R</t>
   </si>
   <si>
-    <t>RMCF0201FT806R</t>
-  </si>
-  <si>
     <t>Stackpole Electronics</t>
   </si>
   <si>
@@ -526,9 +513,6 @@
     <t>RES SMD 57.6 OHM 1% 1/10W 0603</t>
   </si>
   <si>
-    <t>RC0603FR-0757R6L</t>
-  </si>
-  <si>
     <t>No NO J pin 50mA 3mm 100MΩ 100000 12V 250gf@±30gf 2.6mm -30℃~+85℃ 0.65mm Black Round Button Brick nogging SPST SMD Tactile Switches ROHS</t>
   </si>
   <si>
@@ -560,12 +544,24 @@
   </si>
   <si>
     <t>SM_Bottom_Board</t>
+  </si>
+  <si>
+    <t>UMK063CG100DTHF</t>
+  </si>
+  <si>
+    <t>MHT136CGCT</t>
+  </si>
+  <si>
+    <t>0201WMF8060TEE</t>
+  </si>
+  <si>
+    <t>CR0603-FX-57R6ELF</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
@@ -1013,7 +1009,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1142,15 +1138,6 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1178,9 +1165,6 @@
     <xf numFmtId="0" fontId="17" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1194,9 +1178,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1250,6 +1231,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1597,7 +1590,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:L43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1625,10 +1618,10 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="50"/>
-      <c r="J1" s="50"/>
-      <c r="K1" s="50"/>
-      <c r="L1" s="50"/>
+      <c r="I1" s="82"/>
+      <c r="J1" s="82"/>
+      <c r="K1" s="82"/>
+      <c r="L1" s="82"/>
     </row>
     <row r="2" spans="1:12" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1639,7 +1632,7 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="45" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="3"/>
@@ -1657,14 +1650,14 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="46" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
-      <c r="L3" s="51"/>
+      <c r="L3" s="83"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1675,14 +1668,14 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="47" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="6"/>
       <c r="I4" s="6"/>
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
-      <c r="L4" s="52"/>
+      <c r="L4" s="84"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1700,7 +1693,7 @@
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
-      <c r="L5" s="52"/>
+      <c r="L5" s="84"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1714,7 +1707,7 @@
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
-      <c r="L6" s="52"/>
+      <c r="L6" s="84"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1728,7 +1721,7 @@
       <c r="I7" s="7"/>
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
-      <c r="L7" s="52"/>
+      <c r="L7" s="84"/>
     </row>
     <row r="8" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1742,7 +1735,7 @@
       <c r="I8" s="7"/>
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
-      <c r="L8" s="52"/>
+      <c r="L8" s="84"/>
     </row>
     <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -1758,7 +1751,7 @@
       <c r="E9" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="F9" s="53" t="s">
+      <c r="F9" s="50" t="s">
         <v>56</v>
       </c>
       <c r="G9" s="29" t="s">
@@ -1768,7 +1761,7 @@
         <v>91</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="J9" s="29" t="s">
         <v>120</v>
@@ -1777,248 +1770,248 @@
         <v>135</v>
       </c>
       <c r="L9" s="29" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
-      <c r="B10" s="54">
+      <c r="B10" s="51">
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
-      <c r="C10" s="55" t="s">
+      <c r="C10" s="52" t="s">
         <v>121</v>
       </c>
-      <c r="D10" s="56" t="s">
+      <c r="D10" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="E10" s="56" t="s">
+      <c r="E10" s="53" t="s">
         <v>36</v>
       </c>
-      <c r="F10" s="57" t="s">
+      <c r="F10" s="54" t="s">
         <v>57</v>
       </c>
-      <c r="G10" s="56" t="s">
+      <c r="G10" s="53" t="s">
         <v>77</v>
       </c>
-      <c r="H10" s="57" t="s">
+      <c r="H10" s="54" t="s">
         <v>92</v>
       </c>
-      <c r="I10" s="56" t="s">
+      <c r="I10" s="53" t="s">
         <v>107</v>
       </c>
-      <c r="J10" s="81">
+      <c r="J10" s="76">
         <v>1</v>
       </c>
-      <c r="K10" s="56">
+      <c r="K10" s="53">
         <f>J10*20</f>
         <v>20</v>
       </c>
-      <c r="L10" s="85"/>
+      <c r="L10" s="80"/>
     </row>
     <row r="11" spans="1:12" ht="24" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
-      <c r="B11" s="58">
+      <c r="B11" s="55">
         <f t="shared" ref="B11:B40" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
-      <c r="C11" s="59" t="s">
+      <c r="C11" s="56" t="s">
         <v>121</v>
       </c>
-      <c r="D11" s="60" t="s">
-        <v>155</v>
-      </c>
-      <c r="E11" s="60" t="s">
+      <c r="D11" s="57" t="s">
+        <v>154</v>
+      </c>
+      <c r="E11" s="57" t="s">
         <v>37</v>
       </c>
-      <c r="F11" s="61" t="s">
+      <c r="F11" s="58" t="s">
         <v>57</v>
       </c>
-      <c r="G11" s="60" t="s">
+      <c r="G11" s="57" t="s">
         <v>78</v>
       </c>
-      <c r="H11" s="61" t="s">
+      <c r="H11" s="58" t="s">
         <v>92</v>
       </c>
-      <c r="I11" s="60" t="s">
+      <c r="I11" s="57" t="s">
         <v>108</v>
       </c>
-      <c r="J11" s="82">
+      <c r="J11" s="77">
         <v>18</v>
       </c>
-      <c r="K11" s="60">
+      <c r="K11" s="57">
         <f t="shared" ref="K11:K41" si="1">J11*20</f>
         <v>360</v>
       </c>
-      <c r="L11" s="60"/>
+      <c r="L11" s="57"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
-      <c r="B12" s="54">
+      <c r="B12" s="51">
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
-      <c r="C12" s="55" t="s">
+      <c r="C12" s="52" t="s">
         <v>121</v>
       </c>
-      <c r="D12" s="56" t="s">
+      <c r="D12" s="53" t="s">
         <v>8</v>
       </c>
-      <c r="E12" s="56" t="s">
-        <v>156</v>
-      </c>
-      <c r="F12" s="57" t="s">
+      <c r="E12" s="53" t="s">
+        <v>155</v>
+      </c>
+      <c r="F12" s="54" t="s">
         <v>132</v>
       </c>
-      <c r="G12" s="56" t="s">
+      <c r="G12" s="53" t="s">
         <v>137</v>
       </c>
-      <c r="H12" s="57" t="s">
+      <c r="H12" s="54" t="s">
         <v>93</v>
       </c>
-      <c r="I12" s="56" t="s">
+      <c r="I12" s="53" t="s">
         <v>109</v>
       </c>
-      <c r="J12" s="81">
+      <c r="J12" s="76">
         <v>1</v>
       </c>
-      <c r="K12" s="56">
+      <c r="K12" s="53">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L12" s="56"/>
+      <c r="L12" s="53"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
-      <c r="B13" s="58">
+      <c r="B13" s="55">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="59" t="s">
+      <c r="C13" s="56" t="s">
         <v>121</v>
       </c>
-      <c r="D13" s="60" t="s">
+      <c r="D13" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="E13" s="60" t="s">
+      <c r="E13" s="57" t="s">
         <v>38</v>
       </c>
-      <c r="F13" s="61" t="s">
+      <c r="F13" s="58" t="s">
         <v>58</v>
       </c>
-      <c r="G13" s="60" t="s">
+      <c r="G13" s="57" t="s">
         <v>79</v>
       </c>
-      <c r="H13" s="61" t="s">
+      <c r="H13" s="58" t="s">
         <v>94</v>
       </c>
-      <c r="I13" s="60" t="s">
+      <c r="I13" s="57" t="s">
         <v>110</v>
       </c>
-      <c r="J13" s="82">
+      <c r="J13" s="77">
         <v>2</v>
       </c>
-      <c r="K13" s="60">
+      <c r="K13" s="57">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="L13" s="60"/>
+      <c r="L13" s="57"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
-      <c r="B14" s="54">
+      <c r="B14" s="51">
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
       </c>
-      <c r="C14" s="55" t="s">
+      <c r="C14" s="52" t="s">
         <v>121</v>
       </c>
-      <c r="D14" s="56" t="s">
+      <c r="D14" s="53" t="s">
         <v>10</v>
       </c>
-      <c r="E14" s="56" t="s">
+      <c r="E14" s="53" t="s">
         <v>39</v>
       </c>
-      <c r="F14" s="57" t="s">
+      <c r="F14" s="54" t="s">
         <v>58</v>
       </c>
-      <c r="G14" s="56" t="s">
+      <c r="G14" s="53" t="s">
         <v>80</v>
       </c>
-      <c r="H14" s="57" t="s">
+      <c r="H14" s="54" t="s">
         <v>95</v>
       </c>
-      <c r="I14" s="56" t="s">
+      <c r="I14" s="53" t="s">
         <v>111</v>
       </c>
-      <c r="J14" s="81">
+      <c r="J14" s="76">
         <v>2</v>
       </c>
-      <c r="K14" s="56">
+      <c r="K14" s="53">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="L14" s="56"/>
+      <c r="L14" s="53"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
-      <c r="B15" s="58">
+      <c r="B15" s="55">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="59" t="s">
+      <c r="C15" s="56" t="s">
         <v>121</v>
       </c>
-      <c r="D15" s="60" t="s">
+      <c r="D15" s="57" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="60" t="s">
-        <v>157</v>
-      </c>
-      <c r="F15" s="61" t="s">
+      <c r="E15" s="57" t="s">
+        <v>156</v>
+      </c>
+      <c r="F15" s="58" t="s">
         <v>59</v>
       </c>
-      <c r="G15" s="62" t="s">
-        <v>158</v>
-      </c>
-      <c r="H15" s="61" t="s">
+      <c r="G15" s="57" t="s">
+        <v>175</v>
+      </c>
+      <c r="H15" s="58" t="s">
         <v>96</v>
       </c>
-      <c r="I15" s="60" t="s">
+      <c r="I15" s="57" t="s">
         <v>112</v>
       </c>
-      <c r="J15" s="82">
+      <c r="J15" s="77">
         <v>2</v>
       </c>
-      <c r="K15" s="60">
+      <c r="K15" s="57">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="L15" s="60"/>
+      <c r="L15" s="57"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
-      <c r="B16" s="58">
+      <c r="B16" s="55">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="63" t="s">
+      <c r="C16" s="59" t="s">
         <v>122</v>
       </c>
       <c r="D16" s="34" t="s">
         <v>144</v>
       </c>
       <c r="E16" s="34" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="F16" s="35" t="s">
         <v>132</v>
       </c>
-      <c r="G16" s="64" t="s">
+      <c r="G16" s="60" t="s">
         <v>138</v>
       </c>
       <c r="H16" s="35" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="I16" s="34" t="s">
         <v>136</v>
@@ -2034,11 +2027,11 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
-      <c r="B17" s="54">
+      <c r="B17" s="51">
         <f>ROW(B17) - ROW($B$9)</f>
         <v>8</v>
       </c>
-      <c r="C17" s="65" t="s">
+      <c r="C17" s="61" t="s">
         <v>122</v>
       </c>
       <c r="D17" s="32" t="s">
@@ -2070,11 +2063,11 @@
     </row>
     <row r="18" spans="1:12" ht="36" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
-      <c r="B18" s="58">
+      <c r="B18" s="55">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C18" s="63" t="s">
+      <c r="C18" s="59" t="s">
         <v>123</v>
       </c>
       <c r="D18" s="34" t="s">
@@ -2106,11 +2099,11 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
-      <c r="B19" s="54">
+      <c r="B19" s="51">
         <f>ROW(B19) - ROW($B$9)</f>
         <v>10</v>
       </c>
-      <c r="C19" s="66" t="s">
+      <c r="C19" s="62" t="s">
         <v>124</v>
       </c>
       <c r="D19" s="32" t="s">
@@ -2142,11 +2135,11 @@
     </row>
     <row r="20" spans="1:12" ht="36" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
-      <c r="B20" s="58">
+      <c r="B20" s="55">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="63" t="s">
+      <c r="C20" s="59" t="s">
         <v>123</v>
       </c>
       <c r="D20" s="34" t="s">
@@ -2178,11 +2171,11 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
-      <c r="B21" s="54">
+      <c r="B21" s="51">
         <f>ROW(B21) - ROW($B$9)</f>
         <v>12</v>
       </c>
-      <c r="C21" s="66" t="s">
+      <c r="C21" s="62" t="s">
         <v>125</v>
       </c>
       <c r="D21" s="32" t="s">
@@ -2194,11 +2187,11 @@
       <c r="F21" s="33" t="s">
         <v>64</v>
       </c>
-      <c r="G21" s="67" t="s">
-        <v>160</v>
+      <c r="G21" s="32" t="s">
+        <v>176</v>
       </c>
       <c r="H21" s="33" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="I21" s="32" t="s">
         <v>136</v>
@@ -2214,11 +2207,11 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
-      <c r="B22" s="58">
+      <c r="B22" s="55">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C22" s="63" t="s">
+      <c r="C22" s="59" t="s">
         <v>126</v>
       </c>
       <c r="D22" s="34" t="s">
@@ -2250,11 +2243,11 @@
     </row>
     <row r="23" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
-      <c r="B23" s="54">
+      <c r="B23" s="51">
         <f>ROW(B23) - ROW($B$9)</f>
         <v>14</v>
       </c>
-      <c r="C23" s="66" t="s">
+      <c r="C23" s="62" t="s">
         <v>127</v>
       </c>
       <c r="D23" s="32" t="s">
@@ -2286,11 +2279,11 @@
     </row>
     <row r="24" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
-      <c r="B24" s="58">
+      <c r="B24" s="55">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C24" s="63" t="s">
+      <c r="C24" s="59" t="s">
         <v>128</v>
       </c>
       <c r="D24" s="34" t="s">
@@ -2322,11 +2315,11 @@
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
-      <c r="B25" s="54">
+      <c r="B25" s="51">
         <f>ROW(B25) - ROW($B$9)</f>
         <v>16</v>
       </c>
-      <c r="C25" s="66" t="s">
+      <c r="C25" s="62" t="s">
         <v>128</v>
       </c>
       <c r="D25" s="32" t="s">
@@ -2358,27 +2351,27 @@
     </row>
     <row r="26" spans="1:12" ht="36" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
-      <c r="B26" s="58">
+      <c r="B26" s="55">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="C26" s="63" t="s">
+      <c r="C26" s="59" t="s">
         <v>128</v>
       </c>
       <c r="D26" s="34" t="s">
         <v>21</v>
       </c>
       <c r="E26" s="34" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="F26" s="35" t="s">
         <v>67</v>
       </c>
-      <c r="G26" s="68" t="s">
-        <v>163</v>
+      <c r="G26" s="34" t="s">
+        <v>177</v>
       </c>
       <c r="H26" s="35" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="I26" s="34" t="s">
         <v>115</v>
@@ -2394,11 +2387,11 @@
     </row>
     <row r="27" spans="1:12" ht="24" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
-      <c r="B27" s="54">
+      <c r="B27" s="51">
         <f>ROW(B27) - ROW($B$9)</f>
         <v>18</v>
       </c>
-      <c r="C27" s="66" t="s">
+      <c r="C27" s="62" t="s">
         <v>128</v>
       </c>
       <c r="D27" s="32" t="s">
@@ -2430,18 +2423,18 @@
     </row>
     <row r="28" spans="1:12" ht="36" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
-      <c r="B28" s="58">
+      <c r="B28" s="55">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="C28" s="63" t="s">
+      <c r="C28" s="59" t="s">
         <v>128</v>
       </c>
       <c r="D28" s="34" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="E28" s="34" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="F28" s="35" t="s">
         <v>68</v>
@@ -2466,24 +2459,24 @@
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
-      <c r="B29" s="54">
+      <c r="B29" s="51">
         <f>ROW(B29) - ROW($B$9)</f>
         <v>20</v>
       </c>
-      <c r="C29" s="66" t="s">
+      <c r="C29" s="62" t="s">
         <v>128</v>
       </c>
       <c r="D29" s="32" t="s">
         <v>23</v>
       </c>
       <c r="E29" s="32" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="F29" s="33" t="s">
         <v>68</v>
       </c>
-      <c r="G29" s="67" t="s">
-        <v>168</v>
+      <c r="G29" s="32" t="s">
+        <v>178</v>
       </c>
       <c r="H29" s="33" t="s">
         <v>95</v>
@@ -2502,11 +2495,11 @@
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
-      <c r="B30" s="58">
+      <c r="B30" s="55">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="C30" s="63" t="s">
+      <c r="C30" s="59" t="s">
         <v>128</v>
       </c>
       <c r="D30" s="34" t="s">
@@ -2538,54 +2531,54 @@
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
-      <c r="B31" s="54">
+      <c r="B31" s="51">
         <f>ROW(B31) - ROW($B$9)</f>
         <v>22</v>
       </c>
-      <c r="C31" s="69" t="s">
+      <c r="C31" s="64" t="s">
         <v>69</v>
       </c>
-      <c r="D31" s="67" t="s">
+      <c r="D31" s="63" t="s">
         <v>24</v>
       </c>
-      <c r="E31" s="67" t="s">
+      <c r="E31" s="63" t="s">
         <v>50</v>
       </c>
-      <c r="F31" s="70" t="s">
+      <c r="F31" s="65" t="s">
         <v>136</v>
       </c>
-      <c r="G31" s="67" t="s">
+      <c r="G31" s="63" t="s">
         <v>69</v>
       </c>
-      <c r="H31" s="70" t="s">
+      <c r="H31" s="65" t="s">
         <v>136</v>
       </c>
-      <c r="I31" s="67" t="s">
+      <c r="I31" s="63" t="s">
         <v>136</v>
       </c>
-      <c r="J31" s="83">
+      <c r="J31" s="78">
         <v>8</v>
       </c>
-      <c r="K31" s="67">
+      <c r="K31" s="63">
         <f t="shared" si="1"/>
         <v>160</v>
       </c>
-      <c r="L31" s="67"/>
+      <c r="L31" s="63"/>
     </row>
     <row r="32" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
-      <c r="B32" s="58">
+      <c r="B32" s="55">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="C32" s="63" t="s">
+      <c r="C32" s="59" t="s">
         <v>129</v>
       </c>
       <c r="D32" s="34" t="s">
         <v>25</v>
       </c>
       <c r="E32" s="34" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="F32" s="35" t="s">
         <v>132</v>
@@ -2594,7 +2587,7 @@
         <v>140</v>
       </c>
       <c r="H32" s="35" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="I32" s="34" t="s">
         <v>136</v>
@@ -2610,24 +2603,24 @@
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
-      <c r="B33" s="54">
+      <c r="B33" s="51">
         <f>ROW(B33) - ROW($B$9)</f>
         <v>24</v>
       </c>
-      <c r="C33" s="66" t="s">
+      <c r="C33" s="62" t="s">
         <v>130</v>
       </c>
       <c r="D33" s="32" t="s">
         <v>26</v>
       </c>
       <c r="E33" s="32" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F33" s="33" t="s">
         <v>133</v>
       </c>
-      <c r="G33" s="67" t="s">
-        <v>171</v>
+      <c r="G33" s="81" t="s">
+        <v>166</v>
       </c>
       <c r="H33" s="33" t="s">
         <v>102</v>
@@ -2642,29 +2635,27 @@
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L33" s="49" t="s">
-        <v>149</v>
-      </c>
+      <c r="L33" s="49"/>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
-      <c r="B34" s="58">
+      <c r="B34" s="55">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="C34" s="63" t="s">
+      <c r="C34" s="59" t="s">
         <v>130</v>
       </c>
       <c r="D34" s="34" t="s">
         <v>27</v>
       </c>
       <c r="E34" s="34" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="F34" s="35" t="s">
         <v>70</v>
       </c>
-      <c r="G34" s="64" t="s">
+      <c r="G34" s="60" t="s">
         <v>141</v>
       </c>
       <c r="H34" s="35" t="s">
@@ -2684,27 +2675,27 @@
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
-      <c r="B35" s="54">
+      <c r="B35" s="51">
         <f>ROW(B35) - ROW($B$9)</f>
         <v>26</v>
       </c>
-      <c r="C35" s="66" t="s">
+      <c r="C35" s="62" t="s">
         <v>130</v>
       </c>
       <c r="D35" s="32" t="s">
         <v>28</v>
       </c>
       <c r="E35" s="32" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="F35" s="33" t="s">
-        <v>174</v>
-      </c>
-      <c r="G35" s="67" t="s">
+        <v>169</v>
+      </c>
+      <c r="G35" s="32" t="s">
         <v>142</v>
       </c>
       <c r="H35" s="33" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="I35" s="32" t="s">
         <v>136</v>
@@ -2720,24 +2711,24 @@
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
-      <c r="B36" s="58">
+      <c r="B36" s="55">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
-      <c r="C36" s="63" t="s">
+      <c r="C36" s="59" t="s">
         <v>130</v>
       </c>
       <c r="D36" s="34" t="s">
         <v>29</v>
       </c>
       <c r="E36" s="34" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="F36" s="35" t="s">
+        <v>152</v>
+      </c>
+      <c r="G36" s="34" t="s">
         <v>153</v>
-      </c>
-      <c r="G36" s="68" t="s">
-        <v>154</v>
       </c>
       <c r="H36" s="35" t="s">
         <v>102</v>
@@ -2756,11 +2747,11 @@
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
-      <c r="B37" s="54">
+      <c r="B37" s="51">
         <f>ROW(B37) - ROW($B$9)</f>
         <v>28</v>
       </c>
-      <c r="C37" s="66" t="s">
+      <c r="C37" s="62" t="s">
         <v>130</v>
       </c>
       <c r="D37" s="32" t="s">
@@ -2792,11 +2783,11 @@
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
-      <c r="B38" s="58">
+      <c r="B38" s="55">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="C38" s="63" t="s">
+      <c r="C38" s="59" t="s">
         <v>130</v>
       </c>
       <c r="D38" s="34" t="s">
@@ -2828,11 +2819,11 @@
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
-      <c r="B39" s="54">
+      <c r="B39" s="51">
         <f>ROW(B39) - ROW($B$9)</f>
         <v>30</v>
       </c>
-      <c r="C39" s="66" t="s">
+      <c r="C39" s="62" t="s">
         <v>130</v>
       </c>
       <c r="D39" s="32" t="s">
@@ -2864,11 +2855,11 @@
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
-      <c r="B40" s="58">
+      <c r="B40" s="55">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="C40" s="63" t="s">
+      <c r="C40" s="59" t="s">
         <v>131</v>
       </c>
       <c r="D40" s="34" t="s">
@@ -2900,53 +2891,53 @@
     </row>
     <row r="41" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
-      <c r="B41" s="71">
+      <c r="B41" s="66">
         <f>ROW(B41) - ROW($B$9)</f>
         <v>32</v>
       </c>
-      <c r="C41" s="72" t="s">
+      <c r="C41" s="67" t="s">
         <v>131</v>
       </c>
-      <c r="D41" s="73" t="s">
+      <c r="D41" s="68" t="s">
         <v>34</v>
       </c>
-      <c r="E41" s="73" t="s">
+      <c r="E41" s="68" t="s">
         <v>55</v>
       </c>
-      <c r="F41" s="74" t="s">
+      <c r="F41" s="69" t="s">
         <v>132</v>
       </c>
-      <c r="G41" s="73" t="s">
+      <c r="G41" s="68" t="s">
         <v>75</v>
       </c>
-      <c r="H41" s="74" t="s">
+      <c r="H41" s="69" t="s">
         <v>106</v>
       </c>
-      <c r="I41" s="73" t="s">
+      <c r="I41" s="68" t="s">
         <v>143</v>
       </c>
-      <c r="J41" s="84">
+      <c r="J41" s="79">
         <v>1</v>
       </c>
-      <c r="K41" s="73">
+      <c r="K41" s="68">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="L41" s="73"/>
+      <c r="L41" s="68"/>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
-      <c r="B42" s="75"/>
-      <c r="C42" s="76"/>
-      <c r="D42" s="77"/>
-      <c r="E42" s="78"/>
-      <c r="F42" s="79"/>
-      <c r="G42" s="80"/>
-      <c r="H42" s="79"/>
-      <c r="I42" s="80"/>
-      <c r="J42" s="80"/>
-      <c r="K42" s="80"/>
-      <c r="L42" s="86"/>
+      <c r="B42" s="70"/>
+      <c r="C42" s="71"/>
+      <c r="D42" s="72"/>
+      <c r="E42" s="73"/>
+      <c r="F42" s="74"/>
+      <c r="G42" s="75"/>
+      <c r="H42" s="74"/>
+      <c r="I42" s="75"/>
+      <c r="J42" s="75"/>
+      <c r="K42" s="75"/>
+      <c r="L42" s="85"/>
     </row>
     <row r="43" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
@@ -2960,7 +2951,7 @@
       <c r="I43" s="9"/>
       <c r="J43" s="9"/>
       <c r="K43" s="9"/>
-      <c r="L43" s="87"/>
+      <c r="L43" s="86"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>